<commit_message>
save avant de basculer le git
</commit_message>
<xml_diff>
--- a/data/seuils.xlsx
+++ b/data/seuils.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnaud\Documents\PlaneFR\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7737401D-8D08-4C39-A7E4-6571C26341A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E523B3-C8E5-496D-8FDD-55429AA89D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="14595" windowHeight="8746" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="212">
   <si>
     <t>N</t>
   </si>
@@ -690,9 +690,6 @@
     <t>GtCO2eq</t>
   </si>
   <si>
-    <t>Conversion (p.hab)</t>
-  </si>
-  <si>
     <t>Unité affichage (p.hab)</t>
   </si>
   <si>
@@ -742,6 +739,18 @@
   </si>
   <si>
     <t>https://ssp.apps.ece.iiasa.ac.at/basic-drivers?type=line-chart&amp;variables=299&amp;regions=251,76&amp;runs=7,8,9,10,11,12&amp;dataHash=1f0c69e4b47fc1&amp;open=true</t>
+  </si>
+  <si>
+    <t>Conversion exiobase</t>
+  </si>
+  <si>
+    <t>Conversion exiobase (p.hab)</t>
+  </si>
+  <si>
+    <t>Conversion budget</t>
+  </si>
+  <si>
+    <t>Conversion budget (p.hab)</t>
   </si>
 </sst>
 </file>
@@ -993,7 +1002,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1070,29 +1079,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="11" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
@@ -1387,7 +1399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C32444-97C3-4A7C-A91C-82059EB528AD}">
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="21.1328125" style="28" customWidth="1"/>
@@ -1403,28 +1415,28 @@
         <v>76</v>
       </c>
       <c r="B1" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>200</v>
+      </c>
+      <c r="D1" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="E1" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="G1" s="17" t="s">
         <v>201</v>
       </c>
-      <c r="D1" s="17" t="s">
-        <v>196</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>197</v>
-      </c>
-      <c r="F1" s="17" t="s">
+      <c r="H1" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="G1" s="17" t="s">
-        <v>202</v>
-      </c>
-      <c r="H1" s="17" t="s">
+      <c r="I1" s="18" t="s">
         <v>199</v>
-      </c>
-      <c r="I1" s="18" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.45">
@@ -1439,10 +1451,10 @@
         <v>1100</v>
       </c>
       <c r="D2" s="28">
-        <v>12.6</v>
+        <v>10.6</v>
       </c>
       <c r="E2" s="28">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="F2" s="28">
         <v>4.5</v>
@@ -1458,11 +1470,11 @@
       </c>
       <c r="K2" s="28">
         <f>(0.258-K3)/K3</f>
-        <v>1.2845755630300952</v>
+        <v>1.7156275560546412</v>
       </c>
       <c r="L2" s="28">
         <f>0.258/K3</f>
-        <v>2.2845755630300952</v>
+        <v>2.7156275560546415</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.45">
@@ -1477,7 +1489,10 @@
         <v>4500</v>
       </c>
       <c r="D3" s="28">
-        <v>16.399999999999999</v>
+        <v>14.6</v>
+      </c>
+      <c r="E3" s="28">
+        <v>57</v>
       </c>
       <c r="F3" s="28">
         <v>9</v>
@@ -1490,7 +1505,7 @@
       </c>
       <c r="K3" s="28">
         <f>Population!C113*Synthèse!D2/100</f>
-        <v>0.11293126135771475</v>
+        <v>9.5005664316807653E-2</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -1534,60 +1549,86 @@
       <c r="I5" s="20"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A6" s="19"/>
-      <c r="K6" s="28">
+      <c r="A6" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="35"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="35"/>
+      <c r="I6" s="35"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A7" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="B7" s="29">
+        <v>1E-3</v>
+      </c>
+      <c r="C7" s="28">
+        <v>1</v>
+      </c>
+      <c r="D7" s="29">
+        <v>1E-3</v>
+      </c>
+      <c r="E7" s="29">
+        <v>1E-3</v>
+      </c>
+      <c r="F7" s="29">
+        <v>1E-3</v>
+      </c>
+      <c r="G7" s="28">
+        <v>2.7777800000000001E-4</v>
+      </c>
+      <c r="H7" s="29">
+        <v>1E-3</v>
+      </c>
+      <c r="I7" s="29">
+        <v>1</v>
+      </c>
+      <c r="K7" s="28">
         <f>269/100 -1</f>
         <v>1.69</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A7" s="34" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="35"/>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A8" s="34" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="35">
-        <f>((Population!C116/100)*B2)*1000</f>
-        <v>40.756329332322622</v>
+      <c r="B8" s="48">
+        <f>((Population!C123/100)*B2)/B7</f>
+        <v>37.114258799240247</v>
       </c>
       <c r="C8" s="35">
-        <f>(Population!C116/100)*C2</f>
-        <v>8.5081045512042177</v>
+        <f>(Population!C123/100)*C2</f>
+        <v>7.7478025959996817</v>
       </c>
       <c r="D8" s="35">
-        <f>((Population!C116/100)*D2)*1000</f>
-        <v>97.456470313793773</v>
+        <f>((Population!C123/100)*D2)*1000</f>
+        <v>74.660643197815105</v>
       </c>
       <c r="E8" s="35">
-        <f>((Population!C116/100)*E2)*1000</f>
-        <v>440.87450856240042</v>
+        <f>((Population!C123/100)*E2)*1000</f>
+        <v>302.86864693453305</v>
       </c>
       <c r="F8" s="35">
-        <f>((Population!C116/100)*F2)*1000</f>
-        <v>34.805882254926345</v>
+        <f>((Population!C123/100)*F2)*1000</f>
+        <v>31.695556074544147</v>
       </c>
       <c r="G8" s="35">
         <f>(G2*Population!C115)*0.000277778</f>
         <v>738.39512671562909</v>
       </c>
       <c r="H8" s="35">
-        <f>((Population!C116/100)*H2)*1000</f>
-        <v>193.36601252736861</v>
+        <f>((Population!C123/100)*H2)*1000</f>
+        <v>176.08642263635642</v>
       </c>
       <c r="I8" s="35">
-        <f>(Population!C116/100)*I2</f>
-        <v>28.803801226076825</v>
+        <f>(Population!C123/100)*I2</f>
+        <v>26.22983351591165</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.45">
@@ -1595,35 +1636,35 @@
         <v>101</v>
       </c>
       <c r="B9" s="35">
-        <f>((Population!C116/100)*B3)*1000</f>
-        <v>163.78414827574923</v>
+        <f>((Population!C123/100)*B3)*1000</f>
+        <v>149.14805542849609</v>
       </c>
       <c r="C9" s="35">
-        <f>(Population!C116/100)*C3</f>
-        <v>34.805882254926345</v>
+        <f>(Population!C123/100)*C3</f>
+        <v>31.69555607454415</v>
       </c>
       <c r="D9" s="35">
-        <f>((Population!C116/100)*D3)*1000</f>
-        <v>126.84810421795379</v>
+        <f>((Population!C123/100)*D3)*1000</f>
+        <v>102.83447081963213</v>
       </c>
       <c r="E9" s="35">
-        <f>((Population!C116/100)*E3)*1000</f>
-        <v>0</v>
+        <f>((Population!C123/100)*E3)*1000</f>
+        <v>401.47704361089257</v>
       </c>
       <c r="F9" s="35">
-        <f>((Population!C116/100)*F3)*1000</f>
-        <v>69.611764509852691</v>
+        <f>((Population!C123/100)*F3)*1000</f>
+        <v>63.391112149088293</v>
       </c>
       <c r="G9" s="35">
         <f>(G3*Population!C115)*0.000366668</f>
         <v>1206.0487944160323</v>
       </c>
       <c r="H9" s="35">
-        <f>((Population!C116/100)*H3)*1000</f>
-        <v>386.73202505473722</v>
+        <f>((Population!C123/100)*H3)*1000</f>
+        <v>352.17284527271283</v>
       </c>
       <c r="I9" s="35">
-        <f>(Population!C116/100)*I3</f>
+        <f>(Population!C123/100)*I3</f>
         <v>0</v>
       </c>
     </row>
@@ -1669,7 +1710,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A12" s="19" t="s">
-        <v>83</v>
+        <v>208</v>
       </c>
       <c r="B12" s="29">
         <v>1</v>
@@ -1751,299 +1792,329 @@
       <c r="I15" s="22"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="49" t="s">
+        <v>211</v>
+      </c>
+      <c r="B16" s="50">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="C16" s="50">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="D16" s="50">
+        <v>9.9999999999999998E-13</v>
+      </c>
+      <c r="E16" s="50">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="F16" s="50">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="G16" s="50">
+        <v>1</v>
+      </c>
+      <c r="H16" s="50">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="I16" s="50">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A17" s="31" t="s">
         <v>134</v>
       </c>
-      <c r="B16" s="22">
-        <f>B2*1000000000/(Population!B115*1000)</f>
-        <v>0.60715457766544023</v>
-      </c>
-      <c r="C16" s="22">
-        <f>C2*1000000000/(Population!B115*1000)</f>
-        <v>126.74680743201814</v>
-      </c>
-      <c r="D16" s="22">
-        <f>D2*1000000000000/(Population!B115*1000)</f>
-        <v>1451.8270669485714</v>
-      </c>
-      <c r="E16" s="22">
-        <f>E2*1000000000/(Population!B115*1000)</f>
-        <v>6.5677891123863947</v>
-      </c>
-      <c r="F16" s="22">
-        <f>F2*1000000000/(Population!B115*1000)</f>
-        <v>0.51850966676734689</v>
-      </c>
-      <c r="G16" s="22">
+      <c r="B17" s="22">
+        <f>B2*1000000000/(Population!B122*1000)</f>
+        <v>0.54743887261886837</v>
+      </c>
+      <c r="C17" s="22">
+        <f>C2*1000000000/(Population!B122*1000)</f>
+        <v>114.28083048540991</v>
+      </c>
+      <c r="D17" s="22">
+        <f>D2*1000000000000/(Population!B122*1000)</f>
+        <v>1101.2516392230409</v>
+      </c>
+      <c r="E17" s="22">
+        <f>E2*1000000000/(Population!B122*1000)</f>
+        <v>4.4673415553387503</v>
+      </c>
+      <c r="F17" s="22">
+        <f>F2*1000000000/(Population!B122*1000)</f>
+        <v>0.46751248834940412</v>
+      </c>
+      <c r="G17" s="22">
         <f>G2</f>
         <v>39.6</v>
       </c>
-      <c r="H16" s="22">
-        <f>H2*1000000000/(Population!B115*1000)</f>
-        <v>2.8806092598185939</v>
-      </c>
-      <c r="I16" s="22">
-        <f>I2*1000000/(Population!B115*1000)</f>
-        <v>0.42909555534257776</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A17" s="31" t="s">
+      <c r="H17" s="22">
+        <f>H2*1000000000/(Population!B122*1000)</f>
+        <v>2.5972916019411341</v>
+      </c>
+      <c r="I17" s="22">
+        <f>I2*1000000/(Population!B122*1000)</f>
+        <v>0.38689255702515135</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A18" s="31" t="s">
         <v>135</v>
       </c>
-      <c r="B17" s="22">
-        <f>B3*1000000000/(Population!B115*1000)</f>
-        <v>2.4399227556489409</v>
-      </c>
-      <c r="C17" s="22">
-        <f>C3*1000000000/(Population!B115*1000)</f>
-        <v>518.50966676734697</v>
-      </c>
-      <c r="D17" s="22">
-        <f>D3*1000000000000/(Population!B115*1000)</f>
-        <v>1889.6796744409976</v>
-      </c>
-      <c r="E17" s="22">
-        <f>E3*1000000000/(Population!B115*1000)</f>
-        <v>0</v>
-      </c>
-      <c r="F17" s="22">
-        <f>F3*1000000000/(Population!B115*1000)</f>
-        <v>1.0370193335346938</v>
-      </c>
-      <c r="G17" s="22">
+      <c r="B18" s="22">
+        <f>B3*1000000000/(Population!B122*1000)</f>
+        <v>2.1999481050863343</v>
+      </c>
+      <c r="C18" s="22">
+        <f>C3*1000000000/(Population!B122*1000)</f>
+        <v>467.51248834940412</v>
+      </c>
+      <c r="D18" s="22">
+        <f>D3*1000000000000/(Population!B122*1000)</f>
+        <v>1516.8182955336224</v>
+      </c>
+      <c r="E18" s="22">
+        <f>E3*1000000000/(Population!B122*1000)</f>
+        <v>5.9218248524257859</v>
+      </c>
+      <c r="F18" s="22">
+        <f>F3*1000000000/(Population!B122*1000)</f>
+        <v>0.93502497669880824</v>
+      </c>
+      <c r="G18" s="22">
         <f>G3</f>
         <v>49</v>
       </c>
-      <c r="H17" s="22">
-        <f>H3*1000000000/(Population!B115*1000)</f>
-        <v>5.7612185196371879</v>
-      </c>
-      <c r="I17" s="22">
-        <f>I3*1000000/(Population!B115*1000)</f>
+      <c r="H18" s="22">
+        <f>H3*1000000000/(Population!B122*1000)</f>
+        <v>5.1945832038822681</v>
+      </c>
+      <c r="I18" s="22">
+        <f>I3*1000000/(Population!B122*1000)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A18" s="32" t="s">
+    <row r="19" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A19" s="32" t="s">
+        <v>191</v>
+      </c>
+      <c r="B19" s="33" t="s">
         <v>192</v>
       </c>
-      <c r="B18" s="33" t="s">
-        <v>193</v>
-      </c>
-      <c r="C18" s="33" t="s">
+      <c r="C19" s="33" t="s">
         <v>93</v>
       </c>
-      <c r="D18" s="33" t="s">
+      <c r="D19" s="33" t="s">
         <v>94</v>
       </c>
-      <c r="E18" s="33" t="s">
+      <c r="E19" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="F18" s="33" t="s">
+      <c r="F19" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="G18" s="33" t="s">
+      <c r="G19" s="33" t="s">
         <v>92</v>
       </c>
-      <c r="H18" s="33" t="s">
+      <c r="H19" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="I18" s="33" t="s">
+      <c r="I19" s="33" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A19" s="19" t="s">
-        <v>191</v>
-      </c>
-      <c r="B19" s="45">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A20" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="B20" s="45">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="C19" s="45">
+      <c r="C20" s="45">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="D19" s="45">
+      <c r="D20" s="45">
         <v>9.9999999999999995E-7</v>
       </c>
-      <c r="E19" s="45">
+      <c r="E20" s="45">
         <v>1.0000000000000001E-9</v>
       </c>
-      <c r="F19" s="45">
+      <c r="F20" s="45">
         <v>1.0000000000000001E-9</v>
       </c>
-      <c r="G19" s="45">
+      <c r="G20" s="45">
         <v>1E-3</v>
       </c>
-      <c r="H19" s="45">
+      <c r="H20" s="45">
         <v>1E-3</v>
       </c>
-      <c r="I19" s="45">
+      <c r="I20" s="45">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A20" s="19"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="20"/>
-    </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A21" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B21" s="28">
-        <f>(Capacité!G43/100)*B2</f>
-        <v>2.7787518571914371E-3</v>
-      </c>
-      <c r="C21" s="28">
-        <f>(Capacité!G43/100)*C2</f>
-        <v>0.58007950446332146</v>
-      </c>
-      <c r="D21" s="28">
-        <f>(Capacité!G43/100)*D2</f>
-        <v>6.6445470511253182E-3</v>
-      </c>
-      <c r="E21" s="28">
-        <f>(Capacité!G43/100)*E2</f>
-        <v>3.0058665231281204E-2</v>
-      </c>
-      <c r="F21" s="28">
-        <f>(Capacité!G43/100)*F2</f>
-        <v>2.3730525182590425E-3</v>
-      </c>
-      <c r="G21" s="28">
-        <f>(Capacité!G43/100)*G2</f>
-        <v>2.0882862160679572E-2</v>
-      </c>
-      <c r="H21" s="28">
-        <f>((Capacité!G42/100)*H2)*1000</f>
-        <v>13.743345116682876</v>
-      </c>
-      <c r="I21" s="28">
-        <f>(Capacité!G43/100)*I2</f>
-        <v>1.963832795110372</v>
-      </c>
+      <c r="A21" s="19"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A22" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="28">
+        <f>(Capacité!C43/100)*B2</f>
+        <v>2.7787518571914371E-3</v>
+      </c>
+      <c r="C22" s="28">
+        <f>(Capacité!C43/100)*C2</f>
+        <v>0.58007950446332146</v>
+      </c>
+      <c r="D22" s="28">
+        <f>(Capacité!C43/100)*D2</f>
+        <v>5.5898570430101885E-3</v>
+      </c>
+      <c r="E22" s="28">
+        <f>(Capacité!C43/100)*E2</f>
+        <v>2.2675835174475294E-2</v>
+      </c>
+      <c r="F22" s="28">
+        <f>(Capacité!C43/100)*F2</f>
+        <v>2.3730525182590425E-3</v>
+      </c>
+      <c r="G22" s="28">
+        <f>(Capacité!C43/100)*G2</f>
+        <v>2.0882862160679572E-2</v>
+      </c>
+      <c r="H22" s="28">
+        <f>((Capacité!C42/100)*H2)*1000</f>
+        <v>13.743345116682876</v>
+      </c>
+      <c r="I22" s="28">
+        <f>(Capacité!C43/100)*I2</f>
+        <v>1.963832795110372</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A23" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="B22" s="28">
-        <f>(Capacité!G43/100)*B3</f>
+      <c r="B23" s="28">
+        <f>(Capacité!C43/100)*B3</f>
         <v>1.1166744249434098E-2</v>
       </c>
-      <c r="C22" s="28">
-        <f>(Capacité!G43/100)*C3</f>
+      <c r="C23" s="28">
+        <f>(Capacité!C43/100)*C3</f>
         <v>2.3730525182590423</v>
       </c>
-      <c r="D22" s="28">
-        <f>(Capacité!G43/100)*D3</f>
-        <v>8.6484580665440649E-3</v>
-      </c>
-      <c r="E22" s="28">
-        <f>(Capacité!G43/100)*E3</f>
+      <c r="D23" s="28">
+        <f>(Capacité!C43/100)*D3</f>
+        <v>7.6992370592404488E-3</v>
+      </c>
+      <c r="E23" s="28">
+        <f>(Capacité!C43/100)*E3</f>
+        <v>3.0058665231281204E-2</v>
+      </c>
+      <c r="F23" s="28">
+        <f>(Capacité!C43/100)*F3</f>
+        <v>4.746105036518085E-3</v>
+      </c>
+      <c r="G23" s="28">
+        <f>(Capacité!C43/100)*G3</f>
+        <v>2.5839905198820682E-2</v>
+      </c>
+      <c r="H23" s="28">
+        <f>((Capacité!C43/100)*H3)*1000</f>
+        <v>26.367250202878246</v>
+      </c>
+      <c r="I23" s="28">
+        <f>(Capacité!C43/100)*I3</f>
         <v>0</v>
       </c>
-      <c r="F22" s="28">
-        <f>(Capacité!G43/100)*F3</f>
-        <v>4.746105036518085E-3</v>
-      </c>
-      <c r="G22" s="28">
-        <f>(Capacité!G43/100)*G3</f>
-        <v>2.5839905198820682E-2</v>
-      </c>
-      <c r="H22" s="28">
-        <f>((Capacité!G43/100)*H3)*1000</f>
-        <v>26.367250202878246</v>
-      </c>
-      <c r="I22" s="28">
-        <f>(Capacité!G43/100)*I3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A23" s="19"/>
-    </row>
-    <row r="24" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A24" s="19" t="s">
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A24" s="19"/>
+    </row>
+    <row r="25" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A25" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="D24" s="15"/>
-    </row>
-    <row r="25" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A25" s="16" t="s">
+      <c r="D25" s="15"/>
+    </row>
+    <row r="26" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A26" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A26" s="19" t="s">
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="15"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A27" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="B26" s="28">
+      <c r="B27" s="28">
         <f>B2*Besoins!B5*1000</f>
         <v>33.599043710798185</v>
       </c>
-      <c r="C26" s="28" t="e">
+      <c r="C27" s="28" t="e">
         <f>C2*Besoins!C5</f>
         <v>#REF!</v>
       </c>
-      <c r="D26" s="28" t="e">
+      <c r="D27" s="28" t="e">
         <f>D2*Besoins!D5*1000</f>
         <v>#REF!</v>
       </c>
-      <c r="H26" s="28">
+      <c r="H27" s="28">
         <f>H2*Besoins!E5*1000</f>
         <v>183.26764541723307</v>
       </c>
-      <c r="I26" s="28" t="e">
+      <c r="I27" s="28" t="e">
         <f>I2*Besoins!G5</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A27" s="19" t="s">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A28" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="B27" s="28">
+      <c r="B28" s="28">
         <f>B3*Besoins!B5*1000</f>
         <v>135.02174624662513</v>
       </c>
-      <c r="C27" s="28" t="e">
+      <c r="C28" s="28" t="e">
         <f>C3*Besoins!C5</f>
         <v>#REF!</v>
       </c>
-      <c r="D27" s="28" t="e">
+      <c r="D28" s="28" t="e">
         <f>D3*Besoins!D5*1000</f>
         <v>#REF!</v>
       </c>
-      <c r="H27" s="28">
+      <c r="H28" s="28">
         <f>H3*Besoins!E5*1000</f>
         <v>366.53529083446614</v>
       </c>
-      <c r="I27" s="28" t="e">
+      <c r="I28" s="28" t="e">
         <f>I3*Besoins!G5</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A28" s="19"/>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A29" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2524,35 +2595,35 @@
         <v>16</v>
       </c>
       <c r="B19">
-        <f>(Capacité!G43/100)*B2</f>
+        <f>(Capacité!C43/100)*B2</f>
         <v>2.7787518571914371E-3</v>
       </c>
       <c r="C19">
-        <f>(Capacité!G43/100)*C2</f>
+        <f>(Capacité!C43/100)*C2</f>
         <v>1.4765660113611818</v>
       </c>
       <c r="D19">
-        <f>(Capacité!G43/100)*D2</f>
+        <f>(Capacité!C43/100)*D2</f>
         <v>6.6445470511253182E-3</v>
       </c>
       <c r="E19">
-        <f>(Capacité!G43/100)*E2</f>
+        <f>(Capacité!C43/100)*E2</f>
         <v>1.5029332615640602E-2</v>
       </c>
       <c r="F19">
-        <f>(Capacité!G43/100)*F2</f>
+        <f>(Capacité!C43/100)*F2</f>
         <v>9.8613515758764645E-4</v>
       </c>
       <c r="G19">
-        <f>(Capacité!G43/100)*G2</f>
+        <f>(Capacité!C43/100)*G2</f>
         <v>2.0882862160679572E-2</v>
       </c>
       <c r="H19">
-        <f>((Capacité!G42/100)*H2)*1000</f>
+        <f>((Capacité!C42/100)*H2)*1000</f>
         <v>13.743345116682876</v>
       </c>
       <c r="I19">
-        <f>(Capacité!G43/100)*I2</f>
+        <f>(Capacité!C43/100)*I2</f>
         <v>1.963832795110372</v>
       </c>
     </row>
@@ -2561,35 +2632,35 @@
         <v>102</v>
       </c>
       <c r="B20">
-        <f>(Capacité!G43/100)*B3</f>
+        <f>(Capacité!C43/100)*B3</f>
         <v>1.1166744249434098E-2</v>
       </c>
       <c r="C20">
-        <f>(Capacité!G43/100)*C3</f>
+        <f>(Capacité!C43/100)*C3</f>
         <v>2.3730525182590423</v>
       </c>
       <c r="D20">
-        <f>(Capacité!G43/100)*D3</f>
+        <f>(Capacité!C43/100)*D3</f>
         <v>8.6484580665440649E-3</v>
       </c>
       <c r="E20">
-        <f>(Capacité!G43/100)*E3</f>
+        <f>(Capacité!C43/100)*E3</f>
         <v>1.9880906652970199E-2</v>
       </c>
       <c r="F20">
-        <f>(Capacité!G43/100)*F3</f>
+        <f>(Capacité!C43/100)*F3</f>
         <v>8.9648650689786048E-3</v>
       </c>
       <c r="G20">
-        <f>(Capacité!G43/100)*G3</f>
+        <f>(Capacité!C43/100)*G3</f>
         <v>2.5839905198820682E-2</v>
       </c>
       <c r="H20">
-        <f>((Capacité!G43/100)*H3)*1000</f>
+        <f>((Capacité!C43/100)*H3)*1000</f>
         <v>26.367250202878246</v>
       </c>
       <c r="I20">
-        <f>(Capacité!G43/100)*I3</f>
+        <f>(Capacité!C43/100)*I3</f>
         <v>13.746829565772604</v>
       </c>
     </row>
@@ -3043,12 +3114,12 @@
       <c r="A18" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="48" t="s">
+      <c r="B18" s="51" t="s">
         <v>99</v>
       </c>
-      <c r="C18" s="49"/>
-      <c r="D18" s="49"/>
-      <c r="E18" s="49"/>
+      <c r="C18" s="52"/>
+      <c r="D18" s="52"/>
+      <c r="E18" s="52"/>
       <c r="F18" s="21" t="s">
         <v>104</v>
       </c>
@@ -3095,13 +3166,13 @@
         <v>76</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D1" s="23" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
@@ -3300,10 +3371,10 @@
       <c r="A18" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="48" t="s">
+      <c r="B18" s="51" t="s">
         <v>99</v>
       </c>
-      <c r="C18" s="49"/>
+      <c r="C18" s="52"/>
       <c r="D18" s="21" t="s">
         <v>104</v>
       </c>
@@ -3330,124 +3401,124 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:21" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="57" t="s">
         <v>115</v>
       </c>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="53" t="s">
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="52" t="s">
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="57" t="s">
         <v>137</v>
       </c>
-      <c r="I2" s="52"/>
-      <c r="J2" s="52"/>
-      <c r="K2" s="53" t="s">
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="58" t="s">
         <v>138</v>
       </c>
-      <c r="L2" s="53"/>
-      <c r="M2" s="56" t="s">
+      <c r="L2" s="58"/>
+      <c r="M2" s="59" t="s">
         <v>139</v>
       </c>
-      <c r="N2" s="54" t="s">
+      <c r="N2" s="53" t="s">
         <v>140</v>
       </c>
-      <c r="O2" s="52" t="s">
+      <c r="O2" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="P2" s="52"/>
-      <c r="Q2" s="52"/>
-      <c r="R2" s="53" t="s">
+      <c r="P2" s="57"/>
+      <c r="Q2" s="57"/>
+      <c r="R2" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="S2" s="53"/>
-      <c r="T2" s="57" t="s">
+      <c r="S2" s="58"/>
+      <c r="T2" s="60" t="s">
         <v>161</v>
       </c>
-      <c r="U2" s="55" t="s">
+      <c r="U2" s="56" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="17.649999999999999" x14ac:dyDescent="0.45">
-      <c r="B3" s="51" t="s">
+      <c r="B3" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="C3" s="51" t="s">
+      <c r="C3" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="D3" s="51" t="s">
+      <c r="D3" s="54" t="s">
         <v>145</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="55" t="s">
         <v>146</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="55" t="s">
         <v>147</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="G3" s="55" t="s">
         <v>148</v>
       </c>
-      <c r="H3" s="51" t="s">
+      <c r="H3" s="54" t="s">
         <v>149</v>
       </c>
-      <c r="I3" s="51" t="s">
+      <c r="I3" s="54" t="s">
         <v>150</v>
       </c>
-      <c r="J3" s="51" t="s">
+      <c r="J3" s="54" t="s">
         <v>151</v>
       </c>
-      <c r="K3" s="50" t="s">
+      <c r="K3" s="55" t="s">
         <v>152</v>
       </c>
-      <c r="L3" s="50" t="s">
+      <c r="L3" s="55" t="s">
         <v>153</v>
       </c>
-      <c r="M3" s="56"/>
-      <c r="N3" s="54"/>
-      <c r="O3" s="51" t="s">
+      <c r="M3" s="59"/>
+      <c r="N3" s="53"/>
+      <c r="O3" s="54" t="s">
         <v>154</v>
       </c>
-      <c r="P3" s="51" t="s">
+      <c r="P3" s="54" t="s">
         <v>155</v>
       </c>
       <c r="Q3" s="36" t="s">
         <v>156</v>
       </c>
-      <c r="R3" s="50" t="s">
+      <c r="R3" s="55" t="s">
         <v>158</v>
       </c>
-      <c r="S3" s="50" t="s">
+      <c r="S3" s="55" t="s">
         <v>159</v>
       </c>
-      <c r="T3" s="57"/>
-      <c r="U3" s="55"/>
+      <c r="T3" s="60"/>
+      <c r="U3" s="56"/>
     </row>
     <row r="4" spans="1:21" ht="38" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="51"/>
-      <c r="C4" s="51"/>
-      <c r="D4" s="51"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="51"/>
-      <c r="I4" s="51"/>
-      <c r="J4" s="51"/>
-      <c r="K4" s="50"/>
-      <c r="L4" s="50"/>
-      <c r="M4" s="56"/>
-      <c r="N4" s="54"/>
-      <c r="O4" s="51"/>
-      <c r="P4" s="51"/>
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54"/>
+      <c r="K4" s="55"/>
+      <c r="L4" s="55"/>
+      <c r="M4" s="59"/>
+      <c r="N4" s="53"/>
+      <c r="O4" s="54"/>
+      <c r="P4" s="54"/>
       <c r="Q4" s="36" t="s">
         <v>157</v>
       </c>
-      <c r="R4" s="50"/>
-      <c r="S4" s="50"/>
-      <c r="T4" s="57"/>
-      <c r="U4" s="55"/>
+      <c r="R4" s="55"/>
+      <c r="S4" s="55"/>
+      <c r="T4" s="60"/>
+      <c r="U4" s="56"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A5" s="28" t="s">
@@ -3522,6 +3593,17 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
     <mergeCell ref="N2:N4"/>
     <mergeCell ref="J3:J4"/>
     <mergeCell ref="K3:K4"/>
@@ -3536,17 +3618,6 @@
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
     <mergeCell ref="T2:T4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F3:F4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -5254,7 +5325,7 @@
     </row>
     <row r="120" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A120" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B120" s="4">
         <f>AVERAGE(B31:B62)</f>
@@ -5334,7 +5405,7 @@
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B127" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -5347,7 +5418,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D8683F5-D89E-4384-A263-C6122D6DA873}">
-  <dimension ref="A1:AK49"/>
+  <dimension ref="A1:AK53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="11.86328125" bestFit="1" customWidth="1"/>
@@ -6436,19 +6507,19 @@
       <c r="D37" s="13"/>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="E38">
+      <c r="A38">
         <v>2015</v>
       </c>
-      <c r="F38">
+      <c r="B38">
         <f>B27</f>
         <v>17868.090856870793</v>
       </c>
-      <c r="G38" s="28">
-        <f t="shared" ref="G38:H38" si="0">C27</f>
+      <c r="C38" s="28">
+        <f>C27</f>
         <v>50682.895358633301</v>
       </c>
-      <c r="H38" s="28">
-        <f t="shared" si="0"/>
+      <c r="D38" s="28">
+        <f>D27</f>
         <v>47490.67459411014</v>
       </c>
       <c r="K38" t="s">
@@ -6456,45 +6527,39 @@
       </c>
     </row>
     <row r="39" spans="1:13" s="28" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="E39" s="28" t="s">
+      <c r="A39" s="28" t="s">
         <v>168</v>
       </c>
-      <c r="F39" s="28">
+      <c r="B39" s="28">
         <v>1</v>
       </c>
-      <c r="G39" s="28">
-        <f>G38/F38</f>
+      <c r="C39" s="28">
+        <f>C38/B38</f>
         <v>2.8365031141054602</v>
       </c>
-      <c r="H39" s="28">
-        <f>H38/F38</f>
+      <c r="D39" s="28">
+        <f>D38/B38</f>
         <v>2.6578482824228877</v>
       </c>
-      <c r="K39" s="58" t="s">
+      <c r="K39" s="61" t="s">
         <v>169</v>
       </c>
-      <c r="L39" s="58"/>
-      <c r="M39" s="58"/>
+      <c r="L39" s="61"/>
+      <c r="M39" s="61"/>
     </row>
     <row r="40" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A40" t="s">
-        <v>64</v>
+      <c r="A40" s="3" t="s">
+        <v>203</v>
       </c>
       <c r="B40">
-        <v>50000</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="F40">
         <f>SUM(F2:F36)/SUM(Population!B2:B36)</f>
         <v>15732.164711604171</v>
       </c>
-      <c r="G40">
+      <c r="C40">
         <f>SUM(G2:G36)/SUM(Population!C2:C36)</f>
         <v>47663.631330163909</v>
       </c>
-      <c r="H40">
+      <c r="D40">
         <f>SUM(H2:H36)/SUM(Population!D2:D36)</f>
         <v>43700.966271954145</v>
       </c>
@@ -6510,18 +6575,18 @@
       </c>
     </row>
     <row r="41" spans="1:13" s="28" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="E41" s="3" t="s">
+      <c r="A41" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="F41" s="28">
+      <c r="B41" s="28">
         <v>1</v>
       </c>
-      <c r="G41" s="28">
-        <f>G40/F40</f>
+      <c r="C41" s="28">
+        <f>C40/B40</f>
         <v>3.0296931289440945</v>
       </c>
-      <c r="H41" s="28">
-        <f>H40/F40</f>
+      <c r="D41" s="28">
+        <f>D40/B40</f>
         <v>2.7778101153314241</v>
       </c>
       <c r="J41" s="28" t="s">
@@ -6538,25 +6603,19 @@
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A42" t="s">
-        <v>65</v>
+      <c r="A42" s="12" t="s">
+        <v>67</v>
       </c>
       <c r="B42">
-        <v>7500</v>
-      </c>
-      <c r="E42" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="F42">
-        <f>1-(F40-B42)/(B40-B42)</f>
+        <f>1-(B40-B53)/(B51-B53)</f>
         <v>0.80630200678578423</v>
       </c>
-      <c r="G42">
-        <f>1-(G40-B42)/(B40-B42)</f>
+      <c r="C42">
+        <f>1-(C40-B53)/(B51-B53)</f>
         <v>5.4973380466731503E-2</v>
       </c>
-      <c r="H42">
-        <f>1-(H40-B42)/(B40-B42)</f>
+      <c r="D42">
+        <f>1-(D40-B53)/(B51-B53)</f>
         <v>0.14821255830696134</v>
       </c>
       <c r="J42" s="28" t="s">
@@ -6573,19 +6632,19 @@
       </c>
     </row>
     <row r="43" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="E43" s="11" t="s">
+      <c r="A43" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="F43" s="10">
-        <f>(Population!B115*Capacité!F42)*100/(Population!B115*Capacité!F42)</f>
+      <c r="B43" s="10">
+        <f>(Population!B115*Capacité!B42)*100/(Population!B115*Capacité!B42)</f>
         <v>100</v>
       </c>
-      <c r="G43" s="10">
-        <f>(Population!C115*Capacité!G42)*100/(Population!B115*Capacité!F42)</f>
+      <c r="C43" s="10">
+        <f>(Population!C115*Capacité!C42)*100/(Population!B115*Capacité!B42)</f>
         <v>5.2734500405756501E-2</v>
       </c>
-      <c r="H43" s="10">
-        <f>(Population!D115*Capacité!H42)*100/(Population!B115*Capacité!F42)</f>
+      <c r="D43" s="10">
+        <f>(Population!D115*Capacité!D42)*100/(Population!B115*Capacité!B42)</f>
         <v>0.93086683696635297</v>
       </c>
       <c r="I43" s="10"/>
@@ -6602,20 +6661,20 @@
         <v>2.5245850802099499</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="E44" s="3" t="s">
+    <row r="44" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A44" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="F44">
-        <f>1-(B27-B42)/(B40-B42)</f>
+      <c r="B44">
+        <f>1-(B27-B53)/(B51-B53)</f>
         <v>0.75604492101480492</v>
       </c>
-      <c r="G44">
-        <f>MAX(1-(C27-B42)/(B40-B42),0)</f>
+      <c r="C44">
+        <f>MAX(1-(C27-B53)/(B51-B53),0)</f>
         <v>0</v>
       </c>
-      <c r="H44">
-        <f>MAX(1-(D27-B42)/(B40-B42),0)</f>
+      <c r="D44">
+        <f>MAX(1-(D27-B53)/(B51-B53),0)</f>
         <v>5.9042950726820198E-2</v>
       </c>
       <c r="J44" s="28" t="s">
@@ -6632,19 +6691,19 @@
       </c>
     </row>
     <row r="45" spans="1:13" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="E45" s="3" t="s">
+      <c r="A45" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="F45">
-        <f>(Population!B115*Capacité!F44)*100/(Population!B115*Capacité!F44)</f>
+      <c r="B45">
+        <f>(Population!B115*Capacité!B44)*100/(Population!B115*Capacité!B44)</f>
         <v>100</v>
       </c>
-      <c r="G45">
-        <f>(Population!C115*Capacité!G44)*100/(Population!B115*Capacité!F44)</f>
+      <c r="C45">
+        <f>(Population!C115*Capacité!C44)*100/(Population!B115*Capacité!B44)</f>
         <v>0</v>
       </c>
-      <c r="H45">
-        <f>(Population!D115*Capacité!H44)*100/(Population!B115*Capacité!F44)</f>
+      <c r="D45">
+        <f>(Population!D115*Capacité!D44)*100/(Population!B115*Capacité!B44)</f>
         <v>0.39547656087185179</v>
       </c>
       <c r="J45" s="28" t="s">
@@ -6679,7 +6738,7 @@
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B47" s="21" t="s">
         <v>62</v>
@@ -6687,7 +6746,7 @@
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B48" s="21" t="s">
         <v>66</v>
@@ -6695,10 +6754,30 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
+        <v>206</v>
+      </c>
+      <c r="B49" s="21" t="s">
         <v>207</v>
       </c>
-      <c r="B49" s="21" t="s">
-        <v>208</v>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A51" t="s">
+        <v>64</v>
+      </c>
+      <c r="B51">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A52" s="28"/>
+      <c r="B52" s="28"/>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A53" t="s">
+        <v>65</v>
+      </c>
+      <c r="B53">
+        <v>7500</v>
       </c>
     </row>
   </sheetData>
@@ -7018,13 +7097,13 @@
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A19">
-        <f>(Capacité!G43/100)*A2</f>
+        <f>(Capacité!C43/100)*A2</f>
         <v>1.2114682525646763E-3</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A20">
-        <f>(Capacité!G43/100)*A3</f>
+        <f>(Capacité!C43/100)*A3</f>
         <v>7.5182294497396079E-3</v>
       </c>
     </row>

</xml_diff>